<commit_message>
made changes in the data files
</commit_message>
<xml_diff>
--- a/data_files/CallLogData.xlsx
+++ b/data_files/CallLogData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python_Selenium_Project\Python-Automation-Project\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B48105A4-8A11-4979-BADE-467CE3F4D50A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09C96B0-7209-42E6-942A-1CA67B9A7FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{668D8257-2180-4A64-82E0-4141F1E60042}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>name</t>
   </si>
@@ -84,12 +84,6 @@
   </si>
   <si>
     <t>Simple</t>
-  </si>
-  <si>
-    <t>muthu</t>
-  </si>
-  <si>
-    <t>error</t>
   </si>
 </sst>
 </file>
@@ -130,7 +124,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -467,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C737D7B-34C2-4FA0-9BDB-3ECCDC4D2028}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
@@ -553,46 +547,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5">
-        <v>7687560984</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6">
-        <v>9878560351</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <v>27</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>